<commit_message>
Include the screenshot method
</commit_message>
<xml_diff>
--- a/src/main/resources/Testdata/BeneficiaryDetails.xlsx
+++ b/src/main/resources/Testdata/BeneficiaryDetails.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>TestDataID</t>
   </si>
@@ -55,21 +55,6 @@
   </si>
   <si>
     <t>BANGLADESHI</t>
-  </si>
-  <si>
-    <t>BD_002</t>
-  </si>
-  <si>
-    <t>Rahim</t>
-  </si>
-  <si>
-    <t>ABC</t>
-  </si>
-  <si>
-    <t>khan</t>
-  </si>
-  <si>
-    <t>Dhaka</t>
   </si>
 </sst>
 </file>
@@ -410,7 +395,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
@@ -472,29 +457,6 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B3">
-        <v>1812345678</v>
-      </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>12</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>